<commit_message>
fix: clear ground items after a lifetime #955
- const table: add time.GROUND_ITEM (3 minutes) and regenerate the C++ and C# models
- game timers: add ground_item_timer, which destroys items and money left on a map past the lifetime, death drops after the warmth time plus the lifetime
- object container: warn when a map runs out of object ids
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -81,7 +81,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -100,6 +100,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -477,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="10.625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -502,6 +503,26 @@
       </c>
       <c r="D1" s="3" t="n">
         <v>0.0006944444444444445</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GROUND_ITEM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TimeSpan</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>0.002083333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -1170,22 +1191,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>MAX_MEMBER</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>uint8</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="0" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add natural HP and MP recovery
- character stat: recover HP every 10s by 0.5% of max scaled by regenerative and MP every 25s by 2% of max, with a per-character on/off switch
- game timers: add recovery_timer running every second on each thread
- const table: add the recovery sheet and regenerate the C++ and C# models
- character builtin and commands: add natural_recovery and the /자연회복 [켜기|끄기] admin command
- integration tests: turn natural recovery off for every bot when a suite starts
</commit_message>
<xml_diff>
--- a/resources/table/const.xlsx
+++ b/resources/table/const.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bulletin" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="script" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reputation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recovery" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -506,17 +507,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>GROUND_ITEM</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>server</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>TimeSpan</t>
         </is>
@@ -716,6 +717,100 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>hp_interval</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>TimeSpan</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="n">
+        <v>0.0001157407407407407</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>hp_rate</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mp_interval</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TimeSpan</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0.0002893518518518518</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mp_rate</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>